<commit_message>
Major update at end of Spring 2026
</commit_message>
<xml_diff>
--- a/Data/MAPhD Assessment.xlsx
+++ b/Data/MAPhD Assessment.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Groves\Documents\Projects\Department\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82317410-37D3-4CF8-98C4-D3F3755C8203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8992830-544A-4878-809D-B7580AAB3B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{132AA7C1-D575-4F12-9EA7-65249E54CFC9}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{132AA7C1-D575-4F12-9EA7-65249E54CFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Comps" sheetId="1" r:id="rId1"/>
     <sheet name="Class Score" sheetId="2" r:id="rId2"/>
     <sheet name="PhD_Research" sheetId="3" r:id="rId3"/>
+    <sheet name="MA_Research" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -74,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="72">
   <si>
     <t>Micro</t>
   </si>
@@ -263,13 +264,40 @@
   </si>
   <si>
     <t>Thesis</t>
+  </si>
+  <si>
+    <t>Shoaib</t>
+  </si>
+  <si>
+    <t>Mohammad</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Emperical</t>
+  </si>
+  <si>
+    <t>Advisor</t>
+  </si>
+  <si>
+    <t>Cheng</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -290,12 +318,6 @@
       <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1722,4 +1744,84 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A432315-A17F-4139-8B58-458730959129}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2">
+        <v>2026</v>
+      </c>
+      <c r="E2">
+        <v>2262</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>4</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>4</v>
+      </c>
+      <c r="K2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>